<commit_message>
added comments and stuff, duals still missing
</commit_message>
<xml_diff>
--- a/U22 Produktionsplan.xlsx
+++ b/U22 Produktionsplan.xlsx
@@ -1,103 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonia/Documents/01 Uni /01 HWR/05 OR/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5881CE4A-0112-F34D-9031-9A75C1818F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" xr2:uid="{AB7C7CB5-CBC9-674E-AD72-B8CD2F9822C8}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Bedarf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feste Kosten </t>
-  </si>
-  <si>
-    <t>Lagerkosten</t>
-  </si>
-  <si>
-    <t>Produktionskosten</t>
-  </si>
-  <si>
-    <t>Erhöhungskosten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verminderungskosten </t>
-  </si>
-  <si>
-    <t>Produktionsmenge</t>
-  </si>
-  <si>
-    <t>Lagerbestand</t>
-  </si>
-  <si>
-    <t>Periode</t>
-  </si>
-  <si>
-    <t>Anzahl Perioden</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -115,7 +59,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -132,28 +76,86 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -473,112 +475,215 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD30E9F2-6453-4444-BE24-E6F89560C5AF}">
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.5" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.83203125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12.5" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14.83203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="17" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="7.5" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="6.6640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="12.5" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="17" bestFit="1" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feste Kosten </t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Produktionskosten</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Lagerkosten</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Erhöhungskosten</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verminderungskosten </t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Anzahl Perioden</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Gesamtkosten für die Änderung des Produktionsniveaus</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Periode</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Bedarf</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Periode</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Lagerbestand</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Periode</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Produktionsmenge</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="B9" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B11" s="5" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="G2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="4" t="s">
+      <c r="B12" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
-        <v>10</v>
-      </c>
-      <c r="B3" s="3">
-        <v>6</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="G12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="3">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="G3" s="6">
-        <v>4</v>
-      </c>
-      <c r="I3" s="5">
-        <v>0</v>
-      </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5">
-        <v>0</v>
-      </c>
-      <c r="L3" s="5"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I4" s="5">
-        <v>1</v>
-      </c>
-      <c r="J4" s="5">
-        <v>10000</v>
-      </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I5" s="5">
-        <v>2</v>
-      </c>
-      <c r="J5" s="5">
-        <v>8000</v>
-      </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I6" s="5">
-        <v>3</v>
-      </c>
-      <c r="J6" s="5">
-        <v>14000</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="I7" s="5">
-        <v>4</v>
-      </c>
-      <c r="J7" s="5">
+      <c r="H12" s="5" t="n">
         <v>20000</v>
       </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added (a, added gesamtkosten to ausgabe
</commit_message>
<xml_diff>
--- a/U22 Produktionsplan.xlsx
+++ b/U22 Produktionsplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-90" yWindow="-90" windowWidth="17460" windowHeight="10260" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelle1" sheetId="1" state="visible" r:id="rId1"/>
@@ -85,7 +85,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -481,7 +481,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="11.5" bestFit="1" customWidth="1" min="2" max="2"/>

</xml_diff>